<commit_message>
Direct Write Excel for MILLING-04 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-04.xlsx
+++ b/FM-MN-07_MILLING-04.xlsx
@@ -1749,7 +1749,11 @@
       <c r="E6" s="20" t="inlineStr"/>
       <c r="F6" s="20" t="inlineStr"/>
       <c r="G6" s="20" t="inlineStr"/>
-      <c r="H6" s="20" t="inlineStr"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="20" t="inlineStr"/>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
@@ -1790,7 +1794,11 @@
       <c r="E7" s="20" t="inlineStr"/>
       <c r="F7" s="20" t="inlineStr"/>
       <c r="G7" s="20" t="inlineStr"/>
-      <c r="H7" s="20" t="inlineStr"/>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="20" t="inlineStr"/>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
@@ -1831,7 +1839,11 @@
       <c r="E8" s="20" t="inlineStr"/>
       <c r="F8" s="20" t="inlineStr"/>
       <c r="G8" s="20" t="inlineStr"/>
-      <c r="H8" s="20" t="inlineStr"/>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="20" t="inlineStr"/>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
@@ -1872,7 +1884,11 @@
       <c r="E9" s="20" t="inlineStr"/>
       <c r="F9" s="20" t="inlineStr"/>
       <c r="G9" s="20" t="inlineStr"/>
-      <c r="H9" s="20" t="inlineStr"/>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="20" t="inlineStr"/>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
@@ -1913,7 +1929,11 @@
       <c r="E10" s="20" t="inlineStr"/>
       <c r="F10" s="20" t="inlineStr"/>
       <c r="G10" s="20" t="inlineStr"/>
-      <c r="H10" s="20" t="inlineStr"/>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="20" t="inlineStr"/>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
@@ -1954,7 +1974,11 @@
       <c r="E11" s="20" t="inlineStr"/>
       <c r="F11" s="20" t="inlineStr"/>
       <c r="G11" s="20" t="inlineStr"/>
-      <c r="H11" s="20" t="inlineStr"/>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="20" t="inlineStr"/>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
@@ -1995,7 +2019,11 @@
       <c r="E12" s="20" t="inlineStr"/>
       <c r="F12" s="20" t="inlineStr"/>
       <c r="G12" s="20" t="inlineStr"/>
-      <c r="H12" s="20" t="inlineStr"/>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I12" s="20" t="inlineStr"/>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
@@ -2036,7 +2064,11 @@
       <c r="E13" s="21" t="inlineStr"/>
       <c r="F13" s="21" t="inlineStr"/>
       <c r="G13" s="21" t="inlineStr"/>
-      <c r="H13" s="21" t="inlineStr"/>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="21" t="inlineStr"/>
       <c r="J13" s="21" t="inlineStr"/>
       <c r="K13" s="21" t="inlineStr"/>
@@ -2077,7 +2109,11 @@
       <c r="E14" s="21" t="inlineStr"/>
       <c r="F14" s="21" t="inlineStr"/>
       <c r="G14" s="21" t="inlineStr"/>
-      <c r="H14" s="21" t="inlineStr"/>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="21" t="inlineStr"/>
       <c r="J14" s="21" t="inlineStr"/>
       <c r="K14" s="21" t="inlineStr"/>
@@ -2118,7 +2154,11 @@
       <c r="E15" s="21" t="inlineStr"/>
       <c r="F15" s="21" t="inlineStr"/>
       <c r="G15" s="21" t="inlineStr"/>
-      <c r="H15" s="21" t="inlineStr"/>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="21" t="inlineStr"/>
       <c r="J15" s="21" t="inlineStr"/>
       <c r="K15" s="21" t="inlineStr"/>
@@ -2159,7 +2199,11 @@
       <c r="E16" s="21" t="inlineStr"/>
       <c r="F16" s="21" t="inlineStr"/>
       <c r="G16" s="21" t="inlineStr"/>
-      <c r="H16" s="21" t="inlineStr"/>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="21" t="inlineStr"/>
       <c r="J16" s="21" t="inlineStr"/>
       <c r="K16" s="21" t="inlineStr"/>
@@ -2194,7 +2238,11 @@
       <c r="E17" s="28" t="inlineStr"/>
       <c r="F17" s="28" t="inlineStr"/>
       <c r="G17" s="28" t="inlineStr"/>
-      <c r="H17" s="28" t="inlineStr"/>
+      <c r="H17" s="32" t="inlineStr">
+        <is>
+          <t>ชาญวิทย์</t>
+        </is>
+      </c>
       <c r="I17" s="28" t="inlineStr"/>
       <c r="J17" s="28" t="inlineStr"/>
       <c r="K17" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-04 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-04.xlsx
+++ b/FM-MN-07_MILLING-04.xlsx
@@ -1754,7 +1754,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr"/>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="20" t="inlineStr"/>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
@@ -1844,7 +1852,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr"/>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
@@ -1889,7 +1901,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr"/>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
@@ -1934,7 +1950,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr"/>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
@@ -1979,7 +1999,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
@@ -2024,7 +2048,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr"/>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
@@ -2069,7 +2097,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="21" t="inlineStr"/>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="21" t="inlineStr"/>
       <c r="K13" s="21" t="inlineStr"/>
       <c r="L13" s="21" t="inlineStr"/>
@@ -2114,7 +2146,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr"/>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J14" s="21" t="inlineStr"/>
       <c r="K14" s="21" t="inlineStr"/>
       <c r="L14" s="21" t="inlineStr"/>
@@ -2159,7 +2195,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I15" s="21" t="inlineStr"/>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J15" s="21" t="inlineStr"/>
       <c r="K15" s="21" t="inlineStr"/>
       <c r="L15" s="21" t="inlineStr"/>
@@ -2204,7 +2244,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I16" s="21" t="inlineStr"/>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J16" s="21" t="inlineStr"/>
       <c r="K16" s="21" t="inlineStr"/>
       <c r="L16" s="21" t="inlineStr"/>
@@ -2243,7 +2287,11 @@
           <t>ชาญวิทย์</t>
         </is>
       </c>
-      <c r="I17" s="28" t="inlineStr"/>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>ขวัญชัย</t>
+        </is>
+      </c>
       <c r="J17" s="28" t="inlineStr"/>
       <c r="K17" s="28" t="inlineStr"/>
       <c r="L17" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-04 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-04.xlsx
+++ b/FM-MN-07_MILLING-04.xlsx
@@ -1759,7 +1759,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr"/>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
       <c r="M6" s="20" t="inlineStr"/>
@@ -1808,7 +1812,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr"/>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
       <c r="M7" s="20" t="inlineStr"/>
@@ -1857,7 +1865,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="20" t="inlineStr"/>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
       <c r="M8" s="20" t="inlineStr"/>
@@ -1906,7 +1918,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr"/>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
       <c r="M9" s="20" t="inlineStr"/>
@@ -1955,7 +1971,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr"/>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
       <c r="M10" s="20" t="inlineStr"/>
@@ -2004,7 +2024,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr"/>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
       <c r="M11" s="20" t="inlineStr"/>
@@ -2053,7 +2077,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J12" s="20" t="inlineStr"/>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
       <c r="M12" s="20" t="inlineStr"/>
@@ -2102,7 +2130,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="21" t="inlineStr"/>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="21" t="inlineStr"/>
       <c r="L13" s="21" t="inlineStr"/>
       <c r="M13" s="21" t="inlineStr"/>
@@ -2151,7 +2183,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J14" s="21" t="inlineStr"/>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="21" t="inlineStr"/>
       <c r="L14" s="21" t="inlineStr"/>
       <c r="M14" s="21" t="inlineStr"/>
@@ -2200,7 +2236,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J15" s="21" t="inlineStr"/>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="21" t="inlineStr"/>
       <c r="L15" s="21" t="inlineStr"/>
       <c r="M15" s="21" t="inlineStr"/>
@@ -2249,7 +2289,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J16" s="21" t="inlineStr"/>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="21" t="inlineStr"/>
       <c r="L16" s="21" t="inlineStr"/>
       <c r="M16" s="21" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MILLING-04 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_MILLING-04.xlsx
+++ b/FM-MN-07_MILLING-04.xlsx
@@ -1765,7 +1765,11 @@
         </is>
       </c>
       <c r="K6" s="20" t="inlineStr"/>
-      <c r="L6" s="20" t="inlineStr"/>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="20" t="inlineStr"/>
       <c r="N6" s="20" t="inlineStr"/>
       <c r="O6" s="20" t="inlineStr"/>
@@ -1818,7 +1822,11 @@
         </is>
       </c>
       <c r="K7" s="20" t="inlineStr"/>
-      <c r="L7" s="20" t="inlineStr"/>
+      <c r="L7" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="20" t="inlineStr"/>
       <c r="N7" s="20" t="inlineStr"/>
       <c r="O7" s="20" t="inlineStr"/>
@@ -1871,7 +1879,11 @@
         </is>
       </c>
       <c r="K8" s="20" t="inlineStr"/>
-      <c r="L8" s="20" t="inlineStr"/>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="20" t="inlineStr"/>
       <c r="N8" s="20" t="inlineStr"/>
       <c r="O8" s="20" t="inlineStr"/>
@@ -1924,7 +1936,11 @@
         </is>
       </c>
       <c r="K9" s="20" t="inlineStr"/>
-      <c r="L9" s="20" t="inlineStr"/>
+      <c r="L9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="20" t="inlineStr"/>
       <c r="N9" s="20" t="inlineStr"/>
       <c r="O9" s="20" t="inlineStr"/>
@@ -1977,7 +1993,11 @@
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr"/>
-      <c r="L10" s="20" t="inlineStr"/>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="20" t="inlineStr"/>
       <c r="N10" s="20" t="inlineStr"/>
       <c r="O10" s="20" t="inlineStr"/>
@@ -2030,7 +2050,11 @@
         </is>
       </c>
       <c r="K11" s="20" t="inlineStr"/>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="20" t="inlineStr"/>
       <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="20" t="inlineStr"/>
@@ -2083,7 +2107,11 @@
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr"/>
-      <c r="L12" s="20" t="inlineStr"/>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M12" s="20" t="inlineStr"/>
       <c r="N12" s="20" t="inlineStr"/>
       <c r="O12" s="20" t="inlineStr"/>
@@ -2136,7 +2164,11 @@
         </is>
       </c>
       <c r="K13" s="21" t="inlineStr"/>
-      <c r="L13" s="21" t="inlineStr"/>
+      <c r="L13" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="21" t="inlineStr"/>
       <c r="N13" s="21" t="inlineStr"/>
       <c r="O13" s="21" t="inlineStr"/>
@@ -2189,7 +2221,11 @@
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr"/>
-      <c r="L14" s="21" t="inlineStr"/>
+      <c r="L14" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="21" t="inlineStr"/>
       <c r="N14" s="21" t="inlineStr"/>
       <c r="O14" s="21" t="inlineStr"/>
@@ -2242,7 +2278,11 @@
         </is>
       </c>
       <c r="K15" s="21" t="inlineStr"/>
-      <c r="L15" s="21" t="inlineStr"/>
+      <c r="L15" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="21" t="inlineStr"/>
       <c r="N15" s="21" t="inlineStr"/>
       <c r="O15" s="21" t="inlineStr"/>
@@ -2295,7 +2335,11 @@
         </is>
       </c>
       <c r="K16" s="21" t="inlineStr"/>
-      <c r="L16" s="21" t="inlineStr"/>
+      <c r="L16" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="21" t="inlineStr"/>
       <c r="N16" s="21" t="inlineStr"/>
       <c r="O16" s="21" t="inlineStr"/>

</xml_diff>